<commit_message>
Refine competitor benchmark dashboard
</commit_message>
<xml_diff>
--- a/Industry data.xlsx
+++ b/Industry data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bajajbroking-my.sharepoint.com/personal/siddhant_sawant_bajajbroking_in/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="142" documentId="8_{B0CD8669-9272-4ACC-B102-8E0D1CAC65E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3AA722BE-CE4F-46BA-A218-0FDC7C53B5CF}"/>
+  <xr:revisionPtr revIDLastSave="150" documentId="8_{B0CD8669-9272-4ACC-B102-8E0D1CAC65E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FF766402-6112-4BAE-A21E-AC76FC1C541A}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{9699F740-2B94-447D-9E4B-153762A7606C}"/>
   </bookViews>
@@ -2438,7 +2438,7 @@
         </row>
         <row r="25">
           <cell r="B25" t="str">
-            <v>Nu Investors Technologies Private Limited (lemonn)</v>
+            <v>Nu Investors Technologies Private Limited</v>
           </cell>
           <cell r="C25" t="str">
             <v>No</v>
@@ -2728,7 +2728,7 @@
         </row>
         <row r="35">
           <cell r="B35" t="str">
-            <v>Moneywise Finvest Limited (Stoxkart)</v>
+            <v>Moneywise Finvest Limited</v>
           </cell>
           <cell r="C35" t="str">
             <v>No</v>
@@ -3047,7 +3047,7 @@
         </row>
         <row r="46">
           <cell r="B46" t="str">
-            <v>Aaritya Broking Private Ltd (Sahi)</v>
+            <v>Aaritya Broking Private Ltd</v>
           </cell>
           <cell r="C46" t="str">
             <v>No</v>
@@ -3076,7 +3076,7 @@
         </row>
         <row r="47">
           <cell r="B47" t="str">
-            <v>Indusind Securities (Reliance Securities Limited)</v>
+            <v>Indusind Securities Limited (formerly Known As Reliance Securities Limited)</v>
           </cell>
           <cell r="C47" t="str">
             <v>No</v>
@@ -4439,7 +4439,7 @@
         </row>
         <row r="94">
           <cell r="B94" t="str">
-            <v>South Asian Stocks Ltd. (incredstocko.in)</v>
+            <v>South Asian Stocks Ltd.</v>
           </cell>
           <cell r="C94" t="str">
             <v>No</v>
@@ -15210,7 +15210,6 @@
         <v>252951</v>
       </c>
       <c r="G20" s="49">
-        <f>VLOOKUP(TRIM(A20),[1]isc_report1C_2627_300926!$B$10:$J$272,9,FALSE)</f>
         <v>281028</v>
       </c>
       <c r="H20" s="58">
@@ -15482,7 +15481,6 @@
         <v>134637</v>
       </c>
       <c r="G29" s="49">
-        <f>VLOOKUP(TRIM(A29),[1]isc_report1C_2627_300926!$B$10:$J$272,9,FALSE)</f>
         <v>152255</v>
       </c>
       <c r="H29" s="58">
@@ -15762,7 +15760,6 @@
         <v>80710</v>
       </c>
       <c r="G39" s="49">
-        <f>VLOOKUP(TRIM(A39),[1]isc_report1C_2627_300926!$B$10:$J$272,9,FALSE)</f>
         <v>81373</v>
       </c>
       <c r="H39" s="58">
@@ -16238,7 +16235,6 @@
         <v>48869</v>
       </c>
       <c r="G56" s="49">
-        <f>VLOOKUP(TRIM(A56),[1]isc_report1C_2627_300926!$B$10:$J$272,9,FALSE)</f>
         <v>48610</v>
       </c>
       <c r="H56" s="58">
@@ -16322,7 +16318,6 @@
         <v>41057</v>
       </c>
       <c r="G59" s="49">
-        <f>VLOOKUP(TRIM(A59),[1]isc_report1C_2627_300926!$B$10:$J$272,9,FALSE)</f>
         <v>44365</v>
       </c>
       <c r="H59" s="58">
@@ -20430,7 +20425,6 @@
         <v>44925108</v>
       </c>
       <c r="G206" s="60">
-        <f>SUM(G4:G201)</f>
         <v>45080318</v>
       </c>
       <c r="H206" s="35"/>

</xml_diff>

<commit_message>
Refine competition Page with Financials
</commit_message>
<xml_diff>
--- a/Industry data.xlsx
+++ b/Industry data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bajajbroking-my.sharepoint.com/personal/siddhant_sawant_bajajbroking_in/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\siddhantsawant\Downloads\Strategy Tool\competitor-benchmark\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="150" documentId="8_{B0CD8669-9272-4ACC-B102-8E0D1CAC65E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FF766402-6112-4BAE-A21E-AC76FC1C541A}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCC59049-1129-4BEE-884A-89DFD225B374}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{9699F740-2B94-447D-9E4B-153762A7606C}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="4" xr2:uid="{9699F740-2B94-447D-9E4B-153762A7606C}"/>
   </bookViews>
   <sheets>
     <sheet name="Broking data" sheetId="1" r:id="rId1"/>
@@ -22,6 +22,7 @@
   </sheets>
   <externalReferences>
     <externalReference r:id="rId7"/>
+    <externalReference r:id="rId8"/>
   </externalReferences>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'NSE active client data'!$A$2:$J$2</definedName>
@@ -68,8 +69,32 @@
 </comments>
 </file>
 
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={5A1865E8-B5F1-4437-BB1E-C4BC5624C76F}</author>
+  </authors>
+  <commentList>
+    <comment ref="L16" authorId="0" shapeId="0" xr:uid="{5A1865E8-B5F1-4437-BB1E-C4BC5624C76F}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+[Tasks]
+There is a task anchored to this comment that cannot be viewed in your client.
+Comment:
+    @Siddhant Sawant 3% kaa se aaya. Also sae tat note forbakup.
+Reply:
+    It will come in others, had not completed it. Now did it and yes will add that note for backup
+Reply:
+    Ok thanks</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="562" uniqueCount="310">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="607" uniqueCount="333">
   <si>
     <t>Source</t>
   </si>
@@ -980,32 +1005,102 @@
     <t>SIP AUM (In Cr)</t>
   </si>
   <si>
-    <t>Company</t>
-  </si>
-  <si>
     <t>Groww</t>
   </si>
   <si>
-    <t>ROCE</t>
-  </si>
-  <si>
     <t>ROE</t>
   </si>
   <si>
-    <t>CATEGORY</t>
-  </si>
-  <si>
-    <t>Tech-Drive</t>
-  </si>
-  <si>
     <t>Zerodha</t>
+  </si>
+  <si>
+    <t>FY26</t>
+  </si>
+  <si>
+    <t>Tech Driven Brokers</t>
+  </si>
+  <si>
+    <t>Traditional Brokers</t>
+  </si>
+  <si>
+    <t>Angel One</t>
+  </si>
+  <si>
+    <t>Bajaj Broking</t>
+  </si>
+  <si>
+    <t>Motilal</t>
+  </si>
+  <si>
+    <t>ICICI Sec</t>
+  </si>
+  <si>
+    <t>HDFC Sec</t>
+  </si>
+  <si>
+    <t>Kotak Sec</t>
+  </si>
+  <si>
+    <t>Total Revenue</t>
+  </si>
+  <si>
+    <t>PAT</t>
+  </si>
+  <si>
+    <t>opening networth</t>
+  </si>
+  <si>
+    <t>Networth</t>
+  </si>
+  <si>
+    <t>closing net worth</t>
+  </si>
+  <si>
+    <t>Avg Networth</t>
+  </si>
+  <si>
+    <t>MTF book</t>
+  </si>
+  <si>
+    <t>Revenue Mix</t>
+  </si>
+  <si>
+    <t>Equity Derivatives (F&amp;O)</t>
+  </si>
+  <si>
+    <t>Broking</t>
+  </si>
+  <si>
+    <t>Stocks (Cash)</t>
+  </si>
+  <si>
+    <t>Commodity Derivatives</t>
+  </si>
+  <si>
+    <t>Distribution/Services</t>
+  </si>
+  <si>
+    <t>MTF</t>
+  </si>
+  <si>
+    <t>MTF/Loan Interest</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MTF </t>
+  </si>
+  <si>
+    <t>DPC</t>
+  </si>
+  <si>
+    <t>Treasury/Interest Income</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="9">
+  <numFmts count="12">
+    <numFmt numFmtId="44" formatCode="_ &quot;₹&quot;\ * #,##0.00_ ;_ &quot;₹&quot;\ * \-#,##0.00_ ;_ &quot;₹&quot;\ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="164" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="165" formatCode="_ * #,##0.0_ ;_ * \-#,##0.0_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
@@ -1015,8 +1110,10 @@
     <numFmt numFmtId="169" formatCode="0.0"/>
     <numFmt numFmtId="170" formatCode="[$-409]d/mmm/yy;@"/>
     <numFmt numFmtId="171" formatCode="[&gt;=10000000]#.###\,##\,##0;[&gt;=100000]#.###\,##0;##,##0.0"/>
+    <numFmt numFmtId="172" formatCode="&quot;₹&quot;\ #,##0.00"/>
+    <numFmt numFmtId="173" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="23" x14ac:knownFonts="1">
+  <fonts count="28" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1157,8 +1254,42 @@
       <color indexed="8"/>
       <name val="Rubik"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1204,6 +1335,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1386,7 +1523,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="161">
+  <cellStyleXfs count="162">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -1550,8 +1687,9 @@
     <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="96">
+  <cellXfs count="142">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1762,8 +1900,120 @@
     <xf numFmtId="4" fontId="20" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="172" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="3" applyFont="1"/>
+    <xf numFmtId="172" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="10" fontId="0" fillId="9" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="172" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="23" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="173" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="161" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="161" applyFont="1"/>
+    <xf numFmtId="173" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="161">
+  <cellStyles count="162">
     <cellStyle name="Comma" xfId="2" builtinId="3"/>
     <cellStyle name="Comma 10 5" xfId="15" xr:uid="{537EED21-785E-48F4-A453-1417CCF62D6D}"/>
     <cellStyle name="Comma 11" xfId="51" xr:uid="{A31B6CD8-098C-4A8D-8D4E-4D6DF514FDB7}"/>
@@ -1878,6 +2128,7 @@
     <cellStyle name="Comma 7 2 4" xfId="152" xr:uid="{9FF2F0B4-7B2F-4039-9F35-03DCC0ED245C}"/>
     <cellStyle name="Comma 8" xfId="99" xr:uid="{05A2EC26-EF02-4F86-B073-404B8641F454}"/>
     <cellStyle name="Comma 9" xfId="142" xr:uid="{DA66A303-E542-4D22-9E64-FAF6256258B8}"/>
+    <cellStyle name="Currency" xfId="161" builtinId="4"/>
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Indian Comma" xfId="25" xr:uid="{6EC22827-C830-4F05-B830-B1D9CA67E242}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1990,11 +2241,45 @@
 </styleSheet>
 </file>
 
+<file path=xl/documenttasks/documenttask1.xml><?xml version="1.0" encoding="utf-8"?>
+<Tasks xmlns="http://schemas.microsoft.com/office/tasks/2019/documenttasks">
+  <Task id="{DCC9742B-ADF0-42D1-8289-62D924E166AA}">
+    <Anchor>
+      <Comment id="{5A1865E8-B5F1-4437-BB1E-C4BC5624C76F}"/>
+    </Anchor>
+    <History>
+      <Event time="2026-10-21T11:25:37.90" id="{B173F471-2C3F-4BA8-915B-7CFCFD43D415}">
+        <Attribution userId="S::prabal.selwadiya@bajajbroking.in::ba547732-48f4-4194-8b68-ec3df1128f3a" userName="Prabal Selwadiya" userProvider="AD"/>
+        <Anchor>
+          <Comment id="{5A1865E8-B5F1-4437-BB1E-C4BC5624C76F}"/>
+        </Anchor>
+        <Create/>
+      </Event>
+      <Event time="2026-10-21T11:25:37.90" id="{8B4513C8-AB87-4B4B-B921-B9C365CCED43}">
+        <Attribution userId="S::prabal.selwadiya@bajajbroking.in::ba547732-48f4-4194-8b68-ec3df1128f3a" userName="Prabal Selwadiya" userProvider="AD"/>
+        <Anchor>
+          <Comment id="{5A1865E8-B5F1-4437-BB1E-C4BC5624C76F}"/>
+        </Anchor>
+        <Assign userId="S::siddhant.sawant@bajajbroking.in::705fb5c3-f8e0-4b2a-9b15-78f09f936f1f" userName="Siddhant Sawant" userProvider="AD"/>
+      </Event>
+      <Event time="2026-10-21T11:25:37.90" id="{481C59A6-CD19-4888-BFEB-7154DF0A1DEB}">
+        <Attribution userId="S::prabal.selwadiya@bajajbroking.in::ba547732-48f4-4194-8b68-ec3df1128f3a" userName="Prabal Selwadiya" userProvider="AD"/>
+        <Anchor>
+          <Comment id="{5A1865E8-B5F1-4437-BB1E-C4BC5624C76F}"/>
+        </Anchor>
+        <SetTitle title="@Siddhant Sawant 3% kaa se aaya. Also sae tat note forbakup."/>
+      </Event>
+    </History>
+  </Task>
+</Tasks>
+</file>
+
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <xxl21:alternateUrls>
       <xxl21:absoluteUrl r:id="rId2"/>
+      <xxl21:relativeUrl r:id="rId3"/>
     </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="isc_report1C_2627_300926"/>
@@ -9634,8 +9919,52 @@
 </externalLink>
 </file>
 
+<file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:relativeUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="Consol"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0" refreshError="1">
+        <row r="6">
+          <cell r="S6">
+            <v>5907.8440733620082</v>
+          </cell>
+        </row>
+        <row r="32">
+          <cell r="S32">
+            <v>0.15717022338137798</v>
+          </cell>
+        </row>
+        <row r="51">
+          <cell r="S51">
+            <v>842.84570941674997</v>
+          </cell>
+        </row>
+        <row r="52">
+          <cell r="S52">
+            <v>778.12631234324999</v>
+          </cell>
+        </row>
+        <row r="53">
+          <cell r="S53">
+            <v>271.37660286208001</v>
+          </cell>
+        </row>
+      </sheetData>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Siddhant Sawant" id="{13F8032C-99AB-4D98-B2AF-EA5A9143ECF7}" userId="siddhant.sawant@bajajbroking.in" providerId="PeoplePicker"/>
+  <person displayName="Siddhant Sawant" id="{8C3F3FE3-0318-45BA-87B6-CF039B3E0264}" userId="S::siddhant.sawant@bajajbroking.in::705fb5c3-f8e0-4b2a-9b15-78f09f936f1f" providerId="AD"/>
   <person displayName="Prabal Selwadiya" id="{45E6C18B-D63D-45C7-B049-27FAB2BD2D7A}" userId="S::prabal.selwadiya@bajajbroking.in::ba547732-48f4-4194-8b68-ec3df1128f3a" providerId="AD"/>
 </personList>
 </file>
@@ -9964,6 +10293,23 @@
 </ThreadedComments>
 </file>
 
+<file path=xl/threadedComments/threadedComment2.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="L16" dT="2026-10-21T11:25:37.91" personId="{45E6C18B-D63D-45C7-B049-27FAB2BD2D7A}" id="{5A1865E8-B5F1-4437-BB1E-C4BC5624C76F}">
+    <text>@Siddhant Sawant 3% kaa se aaya. Also sae tat note forbakup.</text>
+    <mentions>
+      <mention mentionpersonId="{13F8032C-99AB-4D98-B2AF-EA5A9143ECF7}" mentionId="{D5684F4C-CE30-48F2-81DA-90710F47F32B}" startIndex="0" length="16"/>
+    </mentions>
+  </threadedComment>
+  <threadedComment ref="L16" dT="2026-10-21T11:34:53.33" personId="{8C3F3FE3-0318-45BA-87B6-CF039B3E0264}" id="{E6D4EE95-46E7-4D47-B525-F1CECFF2106A}" parentId="{5A1865E8-B5F1-4437-BB1E-C4BC5624C76F}">
+    <text>It will come in others, had not completed it. Now did it and yes will add that note for backup</text>
+  </threadedComment>
+  <threadedComment ref="L16" dT="2026-10-21T13:05:03.34" personId="{45E6C18B-D63D-45C7-B049-27FAB2BD2D7A}" id="{534711B7-95D5-416A-BB04-8458892A758D}" parentId="{5A1865E8-B5F1-4437-BB1E-C4BC5624C76F}">
+    <text>Ok thanks</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3EFFFC54-6ABB-4788-81D8-C6029B6E6988}">
   <dimension ref="A1:BO40"/>
@@ -20704,48 +21050,774 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B550A9BB-8240-4E8C-9C06-0026F4160F53}">
-  <dimension ref="A1:D3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B550A9BB-8240-4E8C-9C06-0026F4160F53}">
+  <dimension ref="A1:Q29"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.1796875" customWidth="1"/>
+    <col min="3" max="4" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11" customWidth="1"/>
+    <col min="6" max="6" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.81640625" customWidth="1"/>
+    <col min="8" max="8" width="15.81640625" customWidth="1"/>
+    <col min="9" max="9" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.90625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="12.6328125" bestFit="1" customWidth="1"/>
+    <col min="20" max="22" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="10.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A1" s="96" t="s">
+        <v>306</v>
+      </c>
+      <c r="B1" s="96"/>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="C2" s="97" t="s">
         <v>307</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D2" s="97"/>
+      <c r="E2" s="98"/>
+      <c r="F2" s="98"/>
+      <c r="G2" s="98"/>
+      <c r="J2" s="97" t="s">
+        <v>308</v>
+      </c>
+      <c r="K2" s="97"/>
+      <c r="L2" s="97"/>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="C3" s="99" t="s">
         <v>303</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D3" s="99" t="s">
+        <v>309</v>
+      </c>
+      <c r="E3" s="99" t="s">
         <v>305</v>
       </c>
-      <c r="D1" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>308</v>
-      </c>
-      <c r="B2" t="s">
+      <c r="F3" s="99" t="s">
+        <v>310</v>
+      </c>
+      <c r="G3" s="100"/>
+      <c r="H3" s="101"/>
+      <c r="I3" s="99" t="s">
+        <v>311</v>
+      </c>
+      <c r="J3" s="99" t="s">
+        <v>312</v>
+      </c>
+      <c r="K3" s="99" t="s">
+        <v>313</v>
+      </c>
+      <c r="L3" s="99" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A4" s="102" t="s">
+        <v>315</v>
+      </c>
+      <c r="C4" s="103">
+        <v>4644.5</v>
+      </c>
+      <c r="D4" s="104">
+        <v>5072</v>
+      </c>
+      <c r="E4" s="103">
+        <v>7464</v>
+      </c>
+      <c r="F4" s="104">
+        <v>1069.6300000000001</v>
+      </c>
+      <c r="G4" s="104"/>
+      <c r="H4" s="105"/>
+      <c r="I4" s="103">
+        <v>4890</v>
+      </c>
+      <c r="J4" s="103">
+        <v>5889.8</v>
+      </c>
+      <c r="K4" s="103">
+        <v>3110.15</v>
+      </c>
+      <c r="L4" s="103">
+        <f>546149.37/100</f>
+        <v>5461.4937</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A5" s="102" t="s">
+        <v>316</v>
+      </c>
+      <c r="C5" s="103">
+        <v>2083</v>
+      </c>
+      <c r="D5" s="104">
+        <v>1022.7</v>
+      </c>
+      <c r="E5" s="103">
+        <v>4283</v>
+      </c>
+      <c r="F5" s="104">
+        <v>202.57</v>
+      </c>
+      <c r="G5" s="104"/>
+      <c r="I5" s="103">
+        <v>922.51</v>
+      </c>
+      <c r="J5" s="103">
+        <v>1713.1</v>
+      </c>
+      <c r="K5" s="103">
+        <v>929.99400000000003</v>
+      </c>
+      <c r="L5" s="103">
+        <v>1664</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="102" t="s">
+        <v>317</v>
+      </c>
+      <c r="C6" s="103">
+        <f>48554.45/10</f>
+        <v>4855.4449999999997</v>
+      </c>
+      <c r="D6" s="104">
+        <f>(55075.74+903)/10</f>
+        <v>5597.8739999999998</v>
+      </c>
+      <c r="E6" s="106">
+        <v>16500</v>
+      </c>
+      <c r="F6" s="104">
+        <v>1288.93</v>
+      </c>
+      <c r="G6" s="104"/>
+      <c r="I6" s="103">
+        <f>711687/100</f>
+        <v>7116.87</v>
+      </c>
+      <c r="J6" s="103">
+        <f>54220.6/10</f>
+        <v>5422.0599999999995</v>
+      </c>
+      <c r="K6" s="103">
+        <v>3348.59</v>
+      </c>
+      <c r="L6" s="103">
+        <f>1000868.33/100</f>
+        <v>10008.683299999999</v>
+      </c>
+      <c r="P6">
+        <v>1049</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="102" t="s">
+        <v>318</v>
+      </c>
+      <c r="B7" s="107" t="s">
+        <v>319</v>
+      </c>
+      <c r="C7" s="103">
+        <v>9651.4000000000015</v>
+      </c>
+      <c r="D7" s="104">
+        <v>6201.9</v>
+      </c>
+      <c r="E7" s="103">
+        <f>E6+E5</f>
+        <v>20783</v>
+      </c>
+      <c r="F7" s="104">
+        <v>2085.9699999999998</v>
+      </c>
+      <c r="G7" s="104"/>
+      <c r="I7" s="103">
+        <v>7950.56</v>
+      </c>
+      <c r="J7" s="103">
+        <v>6294.5</v>
+      </c>
+      <c r="K7" s="103">
+        <v>3595.92</v>
+      </c>
+      <c r="L7" s="103">
+        <v>11614.4</v>
+      </c>
+      <c r="P7">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A8" s="102" t="s">
+        <v>320</v>
+      </c>
+      <c r="B8" s="107"/>
+      <c r="C8" s="103">
+        <f>AVERAGE(C6:C7)</f>
+        <v>7253.4225000000006</v>
+      </c>
+      <c r="D8" s="103">
+        <f t="shared" ref="D8:L8" si="0">AVERAGE(D6:D7)</f>
+        <v>5899.8869999999997</v>
+      </c>
+      <c r="E8" s="103">
+        <f t="shared" si="0"/>
+        <v>18641.5</v>
+      </c>
+      <c r="F8" s="103">
+        <v>1687.45</v>
+      </c>
+      <c r="G8" s="104"/>
+      <c r="H8" s="104"/>
+      <c r="I8" s="103">
+        <f t="shared" si="0"/>
+        <v>7533.7150000000001</v>
+      </c>
+      <c r="J8" s="103">
+        <f t="shared" si="0"/>
+        <v>5858.28</v>
+      </c>
+      <c r="K8" s="103">
+        <f t="shared" si="0"/>
+        <v>3472.2550000000001</v>
+      </c>
+      <c r="L8" s="103">
+        <f t="shared" si="0"/>
+        <v>10811.541649999999</v>
+      </c>
+      <c r="P8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A9" s="102" t="s">
         <v>304</v>
       </c>
-      <c r="C2" s="62">
-        <v>0.373</v>
-      </c>
-      <c r="D2" s="62">
-        <v>0.28799999999999998</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B3" t="s">
+      <c r="C9" s="108">
+        <f>C5/AVERAGE(C6,C7)</f>
+        <v>0.28717477852696432</v>
+      </c>
+      <c r="D9" s="109">
+        <f>D5/AVERAGE(D6:D7)</f>
+        <v>0.17334230299665063</v>
+      </c>
+      <c r="E9" s="108">
+        <f>E5/AVERAGE(E6:E7)</f>
+        <v>0.22975618914786899</v>
+      </c>
+      <c r="F9" s="108">
+        <f>F5/AVERAGE(F6:F7)</f>
+        <v>0.12004503837150732</v>
+      </c>
+      <c r="G9" s="110"/>
+      <c r="I9" s="108">
+        <f>I5/AVERAGE(I6:I7)</f>
+        <v>0.12245087582952102</v>
+      </c>
+      <c r="J9" s="108">
+        <f>J5/AVERAGE(J6:J7)</f>
+        <v>0.29242371481049045</v>
+      </c>
+      <c r="K9" s="108">
+        <f>K5/AVERAGE(K6:K7)</f>
+        <v>0.2678357436305801</v>
+      </c>
+      <c r="L9" s="108">
+        <f>L5/AVERAGE(L6:L7)</f>
+        <v>0.15390959530734455</v>
+      </c>
+      <c r="P9">
+        <f>P6-P7-P8</f>
+        <v>831</v>
+      </c>
+      <c r="Q9" s="105">
+        <f>P9/P6</f>
+        <v>0.79218303145853197</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A10" s="102" t="s">
+        <v>321</v>
+      </c>
+      <c r="C10" s="103">
+        <v>2814.2</v>
+      </c>
+      <c r="D10" s="104">
+        <v>5128</v>
+      </c>
+      <c r="E10" s="106">
+        <v>7000</v>
+      </c>
+      <c r="F10" s="111">
+        <v>7985</v>
+      </c>
+      <c r="I10" s="103">
+        <v>5767.36</v>
+      </c>
+      <c r="J10" s="103">
+        <v>14561.34</v>
+      </c>
+      <c r="K10" s="103">
+        <v>7132.66</v>
+      </c>
+      <c r="L10" s="103">
+        <v>13363.15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="O11" s="104"/>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="B12" s="35"/>
+      <c r="C12" s="112" t="s">
+        <v>303</v>
+      </c>
+      <c r="D12" s="112" t="s">
         <v>309</v>
       </c>
+      <c r="E12" s="112" t="s">
+        <v>305</v>
+      </c>
+      <c r="F12" s="99" t="s">
+        <v>310</v>
+      </c>
+      <c r="G12" s="100"/>
+      <c r="H12" s="101"/>
+      <c r="I12" s="99" t="s">
+        <v>311</v>
+      </c>
+      <c r="J12" s="99" t="s">
+        <v>312</v>
+      </c>
+      <c r="K12" s="99" t="s">
+        <v>313</v>
+      </c>
+      <c r="L12" s="99" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A13" s="113" t="s">
+        <v>322</v>
+      </c>
+      <c r="B13" s="114" t="s">
+        <v>323</v>
+      </c>
+      <c r="C13" s="115">
+        <v>0.55120000000000002</v>
+      </c>
+      <c r="D13" s="116">
+        <v>0.45500000000000002</v>
+      </c>
+      <c r="E13" s="117">
+        <v>0.36699999999999999</v>
+      </c>
+      <c r="F13" s="50">
+        <v>3.0499999999999999E-2</v>
+      </c>
+      <c r="G13" s="50"/>
+      <c r="H13" s="118" t="s">
+        <v>324</v>
+      </c>
+      <c r="I13" s="119">
+        <f t="shared" ref="I13:I19" si="1">P13/$I$4</f>
+        <v>0.15912603524401842</v>
+      </c>
+      <c r="J13" s="120">
+        <v>0.28199999999999997</v>
+      </c>
+      <c r="K13" s="120">
+        <f>1012/K4</f>
+        <v>0.32538623539057598</v>
+      </c>
+      <c r="L13" s="120">
+        <v>0.44</v>
+      </c>
+      <c r="M13" s="121"/>
+      <c r="P13" s="39">
+        <f>[2]Consol!$S$52</f>
+        <v>778.12631234324999</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A14" s="113"/>
+      <c r="B14" s="114" t="s">
+        <v>325</v>
+      </c>
+      <c r="C14" s="115">
+        <v>0.17780000000000001</v>
+      </c>
+      <c r="D14" s="116">
+        <v>8.2500000000000004E-2</v>
+      </c>
+      <c r="E14" s="117"/>
+      <c r="F14" s="50">
+        <v>7.9699999999999993E-2</v>
+      </c>
+      <c r="G14" s="50"/>
+      <c r="H14" s="118"/>
+      <c r="I14" s="119">
+        <f t="shared" si="1"/>
+        <v>0.17236108577029652</v>
+      </c>
+      <c r="J14" s="120"/>
+      <c r="K14" s="120"/>
+      <c r="L14" s="120"/>
+      <c r="N14" s="109"/>
+      <c r="P14" s="39">
+        <f>[2]Consol!$S$51</f>
+        <v>842.84570941674997</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A15" s="113"/>
+      <c r="B15" s="114" t="s">
+        <v>326</v>
+      </c>
+      <c r="C15" s="115">
+        <v>2.3300000000000001E-2</v>
+      </c>
+      <c r="D15" s="122">
+        <v>0.06</v>
+      </c>
+      <c r="E15" s="117"/>
+      <c r="F15" s="50" t="s">
+        <v>132</v>
+      </c>
+      <c r="G15" s="50"/>
+      <c r="H15" s="118"/>
+      <c r="I15" s="119">
+        <f t="shared" si="1"/>
+        <v>5.5496237804106341E-2</v>
+      </c>
+      <c r="J15" s="120"/>
+      <c r="K15" s="120"/>
+      <c r="L15" s="120"/>
+      <c r="M15" s="104"/>
+      <c r="P15" s="39">
+        <f>[2]Consol!$S$53</f>
+        <v>271.37660286208001</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" ht="29" x14ac:dyDescent="0.35">
+      <c r="A16" s="113"/>
+      <c r="B16" s="114" t="s">
+        <v>327</v>
+      </c>
+      <c r="C16" s="115" t="s">
+        <v>132</v>
+      </c>
+      <c r="D16" s="116">
+        <v>3.6999999999999998E-2</v>
+      </c>
+      <c r="E16" s="123" t="s">
+        <v>132</v>
+      </c>
+      <c r="F16" s="50" t="s">
+        <v>132</v>
+      </c>
+      <c r="G16" s="50"/>
+      <c r="H16" s="124" t="s">
+        <v>327</v>
+      </c>
+      <c r="I16" s="119">
+        <f t="shared" si="1"/>
+        <v>0.18988490239522635</v>
+      </c>
+      <c r="J16" s="119">
+        <f>1100/J4</f>
+        <v>0.18676355733641209</v>
+      </c>
+      <c r="K16" s="119">
+        <f>487/K4</f>
+        <v>0.15658408758420012</v>
+      </c>
+      <c r="L16" s="119" t="s">
+        <v>132</v>
+      </c>
+      <c r="M16" s="104"/>
+      <c r="P16" s="39">
+        <f>[2]Consol!$S$32*[2]Consol!$S$6</f>
+        <v>928.5371727126568</v>
+      </c>
+      <c r="Q16" s="105">
+        <f>P16/5000</f>
+        <v>0.18570743454253136</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" ht="29" x14ac:dyDescent="0.35">
+      <c r="A17" s="113"/>
+      <c r="B17" s="114" t="s">
+        <v>328</v>
+      </c>
+      <c r="C17" s="115">
+        <v>6.5199999999999994E-2</v>
+      </c>
+      <c r="D17" s="125">
+        <f>840/D4</f>
+        <v>0.16561514195583596</v>
+      </c>
+      <c r="E17" s="126">
+        <f>448/E4</f>
+        <v>6.0021436227224008E-2</v>
+      </c>
+      <c r="F17" s="50">
+        <v>0.67900000000000005</v>
+      </c>
+      <c r="G17" s="50"/>
+      <c r="H17" s="124" t="s">
+        <v>329</v>
+      </c>
+      <c r="I17" s="119">
+        <f t="shared" si="1"/>
+        <v>0.16012269938650306</v>
+      </c>
+      <c r="J17" s="119">
+        <v>0.26400000000000001</v>
+      </c>
+      <c r="K17" s="119">
+        <f>912.55/K4</f>
+        <v>0.29341028567753963</v>
+      </c>
+      <c r="L17" s="127">
+        <v>0.26</v>
+      </c>
+      <c r="M17" s="128"/>
+      <c r="P17">
+        <f>783</f>
+        <v>783</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A18" s="113"/>
+      <c r="B18" s="114" t="s">
+        <v>331</v>
+      </c>
+      <c r="C18" s="129" t="s">
+        <v>132</v>
+      </c>
+      <c r="D18" s="130"/>
+      <c r="E18" s="126"/>
+      <c r="F18" s="50">
+        <v>3.0800000000000001E-2</v>
+      </c>
+      <c r="G18" s="50"/>
+      <c r="H18" s="124" t="s">
+        <v>331</v>
+      </c>
+      <c r="I18" s="119">
+        <f t="shared" si="1"/>
+        <v>6.0531697341513292E-2</v>
+      </c>
+      <c r="J18" s="119" t="s">
+        <v>132</v>
+      </c>
+      <c r="K18" s="119">
+        <f>45/K4</f>
+        <v>1.4468755526260792E-2</v>
+      </c>
+      <c r="L18" s="131" t="s">
+        <v>132</v>
+      </c>
+      <c r="M18" s="128"/>
+      <c r="P18">
+        <v>296</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" ht="29" x14ac:dyDescent="0.35">
+      <c r="A19" s="113"/>
+      <c r="B19" s="132" t="s">
+        <v>332</v>
+      </c>
+      <c r="C19" s="129">
+        <v>0.1143</v>
+      </c>
+      <c r="D19" s="133">
+        <f>(1619-840)/D4</f>
+        <v>0.15358832807570977</v>
+      </c>
+      <c r="E19" s="134">
+        <f>2269/E4</f>
+        <v>0.30399249732047162</v>
+      </c>
+      <c r="F19" s="50">
+        <v>0.1011</v>
+      </c>
+      <c r="H19" s="124" t="s">
+        <v>332</v>
+      </c>
+      <c r="I19" s="119">
+        <f t="shared" si="1"/>
+        <v>0.10777096114519427</v>
+      </c>
+      <c r="J19" s="119">
+        <v>0.19800000000000001</v>
+      </c>
+      <c r="K19" s="119">
+        <f>585.38/K4-K18</f>
+        <v>0.17374724691735124</v>
+      </c>
+      <c r="L19" s="119">
+        <v>0.21</v>
+      </c>
+      <c r="M19" s="121"/>
+      <c r="P19">
+        <f>1606-P17-P18</f>
+        <v>527</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A20" s="113"/>
+      <c r="B20" s="114" t="s">
+        <v>208</v>
+      </c>
+      <c r="C20" s="115">
+        <v>6.6100000000000006E-2</v>
+      </c>
+      <c r="D20" s="122">
+        <f>1-SUM(D13:D19)</f>
+        <v>4.6296529968454347E-2</v>
+      </c>
+      <c r="E20" s="135">
+        <f>1-SUM(E13:E19)</f>
+        <v>0.26898606645230438</v>
+      </c>
+      <c r="F20" s="50">
+        <v>7.0900000000000005E-2</v>
+      </c>
+      <c r="G20" s="50"/>
+      <c r="H20" s="124" t="s">
+        <v>208</v>
+      </c>
+      <c r="I20" s="136">
+        <f>1-SUM(I13:I19)</f>
+        <v>9.4706380913141763E-2</v>
+      </c>
+      <c r="J20" s="119">
+        <f>1-SUM(J13:J19)</f>
+        <v>6.923644266358786E-2</v>
+      </c>
+      <c r="K20" s="119">
+        <f>1-SUM(K13:K19)</f>
+        <v>3.6403388904072242E-2</v>
+      </c>
+      <c r="L20" s="127">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="C21" s="62"/>
+      <c r="D21" s="62"/>
+      <c r="E21" s="62"/>
+      <c r="F21" s="62"/>
+      <c r="G21" s="62"/>
+      <c r="I21" s="62"/>
+      <c r="J21" s="62"/>
+      <c r="K21" s="62"/>
+      <c r="L21" s="62"/>
+      <c r="M21" s="62"/>
+    </row>
+    <row r="22" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A22" s="96"/>
+      <c r="B22" s="96"/>
+      <c r="E22" s="105"/>
+      <c r="K22" s="104"/>
+    </row>
+    <row r="23" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="C23" s="137"/>
+      <c r="D23" s="137"/>
+      <c r="E23" s="138"/>
+      <c r="F23" s="138"/>
+      <c r="G23" s="138"/>
+      <c r="J23" s="137"/>
+      <c r="K23" s="137"/>
+      <c r="L23" s="137"/>
+    </row>
+    <row r="25" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A25" s="139"/>
+      <c r="B25" s="140"/>
+      <c r="C25" s="62"/>
+      <c r="D25" s="62"/>
+      <c r="E25" s="62"/>
+      <c r="F25" s="62"/>
+      <c r="G25" s="62"/>
+      <c r="I25" s="62"/>
+    </row>
+    <row r="26" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A26" s="139"/>
+      <c r="B26" s="140"/>
+      <c r="C26" s="62"/>
+      <c r="D26" s="62"/>
+      <c r="E26" s="62"/>
+      <c r="F26" s="62"/>
+      <c r="G26" s="62"/>
+      <c r="I26" s="62"/>
+    </row>
+    <row r="27" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A27" s="139"/>
+      <c r="B27" s="140"/>
+      <c r="C27" s="62"/>
+      <c r="D27" s="141"/>
+      <c r="E27" s="62"/>
+      <c r="F27" s="62"/>
+      <c r="G27" s="62"/>
+      <c r="I27" s="62"/>
+    </row>
+    <row r="28" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A28" s="139"/>
+      <c r="B28" s="140"/>
+      <c r="C28" s="62"/>
+      <c r="D28" s="141"/>
+      <c r="E28" s="141"/>
+      <c r="F28" s="141"/>
+      <c r="G28" s="141"/>
+      <c r="I28" s="141"/>
+    </row>
+    <row r="29" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A29" s="139"/>
+      <c r="B29" s="140"/>
+      <c r="C29" s="62"/>
+      <c r="D29" s="62"/>
+      <c r="E29" s="62"/>
+      <c r="F29" s="62"/>
+      <c r="G29" s="62"/>
+      <c r="I29" s="62"/>
     </row>
   </sheetData>
+  <mergeCells count="13">
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="J23:L23"/>
+    <mergeCell ref="A25:A29"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="J2:L2"/>
+    <mergeCell ref="A13:A20"/>
+    <mergeCell ref="E13:E15"/>
+    <mergeCell ref="H13:H15"/>
+    <mergeCell ref="J13:J15"/>
+    <mergeCell ref="K13:K15"/>
+    <mergeCell ref="L13:L15"/>
+    <mergeCell ref="D17:D18"/>
+    <mergeCell ref="E17:E18"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>